<commit_message>
Rectification des noms de fichiers.
</commit_message>
<xml_diff>
--- a/results/resultats_hebdo.xlsx
+++ b/results/resultats_hebdo.xlsx
@@ -571,30 +571,30 @@
         <v>169</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6875</v>
+        <v>0.5</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0625</v>
+        <v>0.125</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>0.375</v>
+        <v>0.3125</v>
       </c>
       <c r="I3" t="n">
-        <v>0.4419417382415922</v>
+        <v>0.2651650429449553</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1286</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
         <v>-0.2173</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>-0.04435</v>
+        <v>-0.10865</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2445882356124268</v>
+        <v>0.1536543035518368</v>
       </c>
       <c r="O3" t="n">
         <v>0.9298319816589355</v>
@@ -602,12 +602,8 @@
       <c r="P3" t="n">
         <v>0.2378971427679062</v>
       </c>
-      <c r="Q3" t="n">
-        <v>0.8470263196161116</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0.6616827507970099</v>
-      </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -633,28 +629,28 @@
         <v>0.55</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5</v>
+        <v>0.5833</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6166666666666667</v>
+        <v>0.6444333333333333</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1607275126832159</v>
+        <v>0.1357496347447511</v>
       </c>
       <c r="J4" t="n">
         <v>0.2983</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1554</v>
+        <v>0.1737</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0274</v>
+        <v>-0.0299</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1603666666666667</v>
+        <v>0.1473666666666667</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1355182767501614</v>
+        <v>0.1656770754610708</v>
       </c>
       <c r="O4" t="n">
         <v>0.9021339416503906</v>
@@ -687,34 +683,34 @@
         <v>209</v>
       </c>
       <c r="E5" t="n">
-        <v>0.75</v>
+        <v>0.7812</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6029</v>
+        <v>0.463</v>
       </c>
       <c r="G5" t="n">
         <v>0.6316000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6615000000000001</v>
+        <v>0.6252666666666666</v>
       </c>
       <c r="I5" t="n">
-        <v>0.07797506011539844</v>
+        <v>0.1591945141433376</v>
       </c>
       <c r="J5" t="n">
-        <v>0.2287</v>
+        <v>0.2572</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1406</v>
+        <v>0.1717</v>
       </c>
       <c r="L5" t="n">
         <v>0.1119</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1604</v>
+        <v>0.1802666666666667</v>
       </c>
       <c r="N5" t="n">
-        <v>0.06086534317655655</v>
+        <v>0.07302782574699408</v>
       </c>
       <c r="O5" t="n">
         <v>0.8454955220222473</v>
@@ -747,34 +743,34 @@
         <v>189</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8929</v>
+        <v>0.8452</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6071</v>
+        <v>0.6795</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6333</v>
+        <v>0.6494</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7111000000000001</v>
+        <v>0.7247</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1579874678574222</v>
+        <v>0.1054357150115652</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2816</v>
+        <v>0.4902</v>
       </c>
       <c r="K6" t="n">
-        <v>0.2377</v>
+        <v>0.2949</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1855</v>
+        <v>0.2196</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2349333333333333</v>
+        <v>0.3349</v>
       </c>
       <c r="N6" t="n">
-        <v>0.04810970103142748</v>
+        <v>0.1396642044333479</v>
       </c>
       <c r="O6" t="n">
         <v>0.6518664360046387</v>
@@ -807,34 +803,34 @@
         <v>182</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7963</v>
+        <v>0.8182</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5222</v>
+        <v>0.6667</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5694</v>
+        <v>0.6786</v>
       </c>
       <c r="H7" t="n">
-        <v>0.6293000000000001</v>
+        <v>0.7211666666666666</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1465391074082274</v>
+        <v>0.08424371390990155</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4683</v>
+        <v>0.3748</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0927</v>
+        <v>0.2856</v>
       </c>
       <c r="L7" t="n">
-        <v>0.0834</v>
+        <v>0.2668</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2148</v>
+        <v>0.3090666666666667</v>
       </c>
       <c r="N7" t="n">
-        <v>0.219586679923897</v>
+        <v>0.05769760249207358</v>
       </c>
       <c r="O7" t="n">
         <v>0.5115828514099121</v>
@@ -867,34 +863,34 @@
         <v>229</v>
       </c>
       <c r="E8" t="n">
+        <v>0.9206</v>
+      </c>
+      <c r="F8" t="n">
         <v>0.7803</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>0.7451</v>
       </c>
-      <c r="G8" t="n">
-        <v>0.7321</v>
-      </c>
       <c r="H8" t="n">
-        <v>0.7524999999999999</v>
+        <v>0.8153333333333332</v>
       </c>
       <c r="I8" t="n">
-        <v>0.02493752192981493</v>
+        <v>0.09284698882211168</v>
       </c>
       <c r="J8" t="n">
+        <v>0.4537</v>
+      </c>
+      <c r="K8" t="n">
         <v>0.3812</v>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>0.3477</v>
       </c>
-      <c r="L8" t="n">
-        <v>0.324</v>
-      </c>
       <c r="M8" t="n">
-        <v>0.3509666666666666</v>
+        <v>0.3941999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>0.02873957782106989</v>
+        <v>0.05418256177037036</v>
       </c>
       <c r="O8" t="n">
         <v>0.6474288702011108</v>
@@ -927,34 +923,34 @@
         <v>99</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7917</v>
+        <v>0.9333</v>
       </c>
       <c r="F9" t="n">
-        <v>0.75</v>
+        <v>0.7083</v>
       </c>
       <c r="G9" t="n">
-        <v>0.625</v>
+        <v>0.8</v>
       </c>
       <c r="H9" t="n">
-        <v>0.7222333333333334</v>
+        <v>0.8138666666666667</v>
       </c>
       <c r="I9" t="n">
-        <v>0.08674942843231494</v>
+        <v>0.1131391326347048</v>
       </c>
       <c r="J9" t="n">
-        <v>0.526</v>
+        <v>0.4835</v>
       </c>
       <c r="K9" t="n">
-        <v>0.2887</v>
+        <v>0.4152</v>
       </c>
       <c r="L9" t="n">
-        <v>0.2582</v>
+        <v>0.3528</v>
       </c>
       <c r="M9" t="n">
-        <v>0.3576333333333333</v>
+        <v>0.4171666666666667</v>
       </c>
       <c r="N9" t="n">
-        <v>0.1466051272409438</v>
+        <v>0.06537219082555924</v>
       </c>
       <c r="O9" t="n">
         <v>0.4962830245494843</v>
@@ -987,34 +983,34 @@
         <v>66</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="F10" t="n">
         <v>0.9</v>
       </c>
       <c r="G10" t="n">
-        <v>0.7778</v>
+        <v>0.5</v>
       </c>
       <c r="H10" t="n">
-        <v>0.8925999999999999</v>
+        <v>0.7666666666666666</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1112846799878581</v>
+        <v>0.2309401076758503</v>
       </c>
       <c r="J10" t="n">
-        <v>0.5774</v>
+        <v>0.5521</v>
       </c>
       <c r="K10" t="n">
-        <v>0.5521</v>
+        <v>0.2057</v>
       </c>
       <c r="L10" t="n">
-        <v>0.3892</v>
+        <v>0.1491</v>
       </c>
       <c r="M10" t="n">
-        <v>0.5062333333333334</v>
+        <v>0.3023</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1021402140850181</v>
+        <v>0.2181763506890699</v>
       </c>
       <c r="O10" t="n">
         <v>0.3117345571517944</v>
@@ -1257,30 +1253,30 @@
         <v>169</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5625</v>
+        <v>0.75</v>
       </c>
       <c r="F3" t="n">
-        <v>0.125</v>
+        <v>0.3125</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>0.34375</v>
+        <v>0.53125</v>
       </c>
       <c r="I3" t="n">
         <v>0.3093592167691145</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0429</v>
+        <v>0.1715</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.2173</v>
+        <v>-0.0639</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>-0.0872</v>
+        <v>0.05380000000000001</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1839891844647397</v>
+        <v>0.1664529362913133</v>
       </c>
       <c r="O3" t="n">
         <v>0.9298319816589355</v>
@@ -1313,34 +1309,34 @@
         <v>207</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9167</v>
+        <v>0.85</v>
       </c>
       <c r="F4" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="G4" t="n">
-        <v>0.45</v>
+        <v>0.5469000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6222333333333333</v>
+        <v>0.7156333333333333</v>
       </c>
       <c r="I4" t="n">
-        <v>0.256238098910629</v>
+        <v>0.1544448229411829</v>
       </c>
       <c r="J4" t="n">
-        <v>0.4684</v>
+        <v>0.4113</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1005</v>
+        <v>0.2691</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0331</v>
+        <v>0.0798</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2006666666666667</v>
+        <v>0.2534</v>
       </c>
       <c r="N4" t="n">
-        <v>0.2343001138141707</v>
+        <v>0.1663067346802288</v>
       </c>
       <c r="O4" t="n">
         <v>0.9021339416503906</v>
@@ -1373,34 +1369,34 @@
         <v>209</v>
       </c>
       <c r="E5" t="n">
-        <v>0.875</v>
+        <v>0.8125</v>
       </c>
       <c r="F5" t="n">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8421</v>
+        <v>0.8158</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8223666666666666</v>
+        <v>0.7594333333333333</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0647943155942968</v>
+        <v>0.09478640901170024</v>
       </c>
       <c r="J5" t="n">
-        <v>0.343</v>
+        <v>0.2858</v>
       </c>
       <c r="K5" t="n">
-        <v>0.2983</v>
+        <v>0.2762</v>
       </c>
       <c r="L5" t="n">
-        <v>0.2911</v>
+        <v>0.2687</v>
       </c>
       <c r="M5" t="n">
-        <v>0.3108</v>
+        <v>0.2769</v>
       </c>
       <c r="N5" t="n">
-        <v>0.02811743231520262</v>
+        <v>0.008571464285639882</v>
       </c>
       <c r="O5" t="n">
         <v>0.8454955220222473</v>
@@ -1433,34 +1429,34 @@
         <v>189</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7077</v>
+        <v>0.7050999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8462</v>
+        <v>0.6591</v>
       </c>
       <c r="G6" t="n">
-        <v>0.4615</v>
+        <v>0.6222</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6718000000000001</v>
+        <v>0.6621333333333332</v>
       </c>
       <c r="I6" t="n">
-        <v>0.194846426705752</v>
+        <v>0.04153315944318867</v>
       </c>
       <c r="J6" t="n">
-        <v>0.354</v>
+        <v>0.4244</v>
       </c>
       <c r="K6" t="n">
-        <v>0.2806</v>
+        <v>0.2313</v>
       </c>
       <c r="L6" t="n">
-        <v>0.0149</v>
+        <v>0.1855</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2165</v>
+        <v>0.2804</v>
       </c>
       <c r="N6" t="n">
-        <v>0.1784063059423629</v>
+        <v>0.1267927837063293</v>
       </c>
       <c r="O6" t="n">
         <v>0.6518664360046387</v>
@@ -1493,34 +1489,34 @@
         <v>182</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7792</v>
+        <v>0.8889</v>
       </c>
       <c r="F7" t="n">
-        <v>0.6914</v>
+        <v>0.7272999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>0.6667</v>
+        <v>0.7917</v>
       </c>
       <c r="H7" t="n">
-        <v>0.7124333333333334</v>
+        <v>0.8026333333333334</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0591258262803433</v>
+        <v>0.08135289382273589</v>
       </c>
       <c r="J7" t="n">
-        <v>0.3367</v>
+        <v>0.4226</v>
       </c>
       <c r="K7" t="n">
-        <v>0.2765</v>
+        <v>0.3153</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1334</v>
+        <v>0.3002</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2488666666666667</v>
+        <v>0.3460333333333334</v>
       </c>
       <c r="N7" t="n">
-        <v>0.1044290349152635</v>
+        <v>0.0667371211046246</v>
       </c>
       <c r="O7" t="n">
         <v>0.5115828514099121</v>
@@ -1553,34 +1549,34 @@
         <v>229</v>
       </c>
       <c r="E8" t="n">
-        <v>0.8038999999999999</v>
+        <v>0.7745</v>
       </c>
       <c r="F8" t="n">
-        <v>0.7411</v>
+        <v>0.7451</v>
       </c>
       <c r="G8" t="n">
-        <v>0.6607</v>
+        <v>0.7321</v>
       </c>
       <c r="H8" t="n">
-        <v>0.7352333333333333</v>
+        <v>0.7505666666666667</v>
       </c>
       <c r="I8" t="n">
-        <v>0.07178003436425294</v>
+        <v>0.02172218527987765</v>
       </c>
       <c r="J8" t="n">
-        <v>0.4196</v>
+        <v>0.3836</v>
       </c>
       <c r="K8" t="n">
-        <v>0.2466</v>
+        <v>0.382</v>
       </c>
       <c r="L8" t="n">
-        <v>0.2287</v>
+        <v>0.3143</v>
       </c>
       <c r="M8" t="n">
-        <v>0.2983</v>
+        <v>0.3599666666666667</v>
       </c>
       <c r="N8" t="n">
-        <v>0.1054294550872762</v>
+        <v>0.03955658394418472</v>
       </c>
       <c r="O8" t="n">
         <v>0.6474288702011108</v>
@@ -1613,34 +1609,34 @@
         <v>99</v>
       </c>
       <c r="E9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F9" t="n">
         <v>0.75</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>1</v>
       </c>
-      <c r="G9" t="n">
-        <v>0.625</v>
-      </c>
       <c r="H9" t="n">
-        <v>0.7916666666666666</v>
+        <v>0.8833333333333333</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1909406539564933</v>
+        <v>0.1258305739211792</v>
       </c>
       <c r="J9" t="n">
+        <v>0.4811</v>
+      </c>
+      <c r="K9" t="n">
         <v>0.3599</v>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>0.3273</v>
       </c>
-      <c r="L9" t="n">
-        <v>0.2981</v>
-      </c>
       <c r="M9" t="n">
-        <v>0.3284333333333334</v>
+        <v>0.3894333333333333</v>
       </c>
       <c r="N9" t="n">
-        <v>0.0309155839882305</v>
+        <v>0.08104179991420069</v>
       </c>
       <c r="O9" t="n">
         <v>0.4962830245494843</v>
@@ -1673,34 +1669,34 @@
         <v>66</v>
       </c>
       <c r="E10" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>0.4333333333333333</v>
+        <v>0.9666666666666667</v>
       </c>
       <c r="I10" t="n">
-        <v>0.3785938897200182</v>
+        <v>0.05773502691896256</v>
       </c>
       <c r="J10" t="n">
-        <v>0.276</v>
+        <v>0.5774</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1155</v>
+        <v>0.5521</v>
       </c>
       <c r="L10" t="n">
-        <v>0.0563</v>
+        <v>0.4472</v>
       </c>
       <c r="M10" t="n">
-        <v>0.1492666666666667</v>
+        <v>0.5255666666666667</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1136756936786987</v>
+        <v>0.0690363913695765</v>
       </c>
       <c r="O10" t="n">
         <v>0.3117345571517944</v>

</xml_diff>